<commit_message>
Fix public pool import feedback and missing address handling
</commit_message>
<xml_diff>
--- a/backend/templates/customer-import-template.xlsx
+++ b/backend/templates/customer-import-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="客户导入模板" sheetId="1" r:id="R743f02971fcd4a4a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="2" r:id="Rbed6ec0ab9024a60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="客户导入模板" sheetId="1" r:id="R7456114a9a954478"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="2" r:id="Rb80766b3251342d5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17530,7 +17530,7 @@
         <x:v>客户地址</x:v>
       </x:c>
       <x:c r="B8" s="23" t="str">
-        <x:v>建议填写完整省市区和街道；导入公海时必填，用于地图生成待拜访灰点。</x:v>
+        <x:v>建议填写完整省市区和街道；公海可先留空，系统会标记待补地址，暂不显示地图灰点。</x:v>
       </x:c>
     </x:row>
     <x:row r="9">

</xml_diff>

<commit_message>
Complete CRM public pool import audit and city improvements
</commit_message>
<xml_diff>
--- a/backend/templates/customer-import-template.xlsx
+++ b/backend/templates/customer-import-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="客户导入模板" sheetId="1" r:id="R7456114a9a954478"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="2" r:id="Rb80766b3251342d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="客户导入模板" sheetId="1" r:id="R177b8a4335764892"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="2" r:id="Rea485a14889b4370"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -205,9 +205,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -359,10 +359,10 @@
   <x:cols>
     <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="17" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="13" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="34" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="15" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="15" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="13" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="34" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="15" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="18" hidden="0" customWidth="1"/>
@@ -382,16 +382,16 @@
         <x:v>客户电话</x:v>
       </x:c>
       <x:c r="C1" s="5" t="str">
+        <x:v>渠道来源</x:v>
+      </x:c>
+      <x:c r="D1" s="5" t="str">
         <x:v>状态</x:v>
       </x:c>
-      <x:c r="D1" s="5" t="str">
+      <x:c r="E1" s="5" t="str">
         <x:v>城市</x:v>
       </x:c>
-      <x:c r="E1" s="5" t="str">
+      <x:c r="F1" s="5" t="str">
         <x:v>客户地址</x:v>
-      </x:c>
-      <x:c r="F1" s="5" t="str">
-        <x:v>渠道来源</x:v>
       </x:c>
       <x:c r="G1" s="5" t="str">
         <x:v>意向产品</x:v>
@@ -429,16 +429,16 @@
         <x:v>13800138000</x:v>
       </x:c>
       <x:c r="C2" s="11" t="str">
+        <x:v>企查查</x:v>
+      </x:c>
+      <x:c r="D2" s="11" t="str">
         <x:v>名单</x:v>
       </x:c>
-      <x:c r="D2" s="11" t="str">
+      <x:c r="E2" s="15" t="str">
         <x:v>杭州市</x:v>
       </x:c>
-      <x:c r="E2" s="15" t="str">
+      <x:c r="F2" s="11" t="str">
         <x:v>浙江省杭州市余杭区示例路88号</x:v>
-      </x:c>
-      <x:c r="F2" s="11" t="str">
-        <x:v>企查查</x:v>
       </x:c>
       <x:c r="G2" s="11" t="str">
         <x:v>V1</x:v>
@@ -476,30 +476,30 @@
         <x:v>13900139000</x:v>
       </x:c>
       <x:c r="C3" s="11" t="str">
+        <x:v>公众号</x:v>
+      </x:c>
+      <x:c r="D3" s="11" t="str">
         <x:v>公海</x:v>
       </x:c>
-      <x:c r="D3" s="11" t="str">
+      <x:c r="E3" s="15" t="str">
         <x:v>佛山市</x:v>
       </x:c>
-      <x:c r="E3" s="15" t="str">
+      <x:c r="F3" s="11" t="str">
         <x:v>广东省佛山市顺德区示例工业园</x:v>
-      </x:c>
-      <x:c r="F3" s="11" t="str">
-        <x:v>公众号</x:v>
       </x:c>
       <x:c r="G3" s="11" t="str">
         <x:v>ERP</x:v>
       </x:c>
-      <x:c r="H3" s="11" t="str"/>
+      <x:c r="H3" s="11"/>
       <x:c r="I3" s="11" t="str">
         <x:v>运营小组</x:v>
       </x:c>
-      <x:c r="J3" s="11" t="str"/>
+      <x:c r="J3" s="11"/>
       <x:c r="K3" s="15" t="str">
         <x:v>自主注册资源，导入公海待认领</x:v>
       </x:c>
-      <x:c r="L3" s="13" t="str"/>
-      <x:c r="M3" s="13" t="str"/>
+      <x:c r="L3" s="13"/>
+      <x:c r="M3" s="13"/>
       <x:c r="N3" s="11" t="str">
         <x:v>云熙</x:v>
       </x:c>
@@ -17459,10 +17459,10 @@
   </x:sheetData>
   <x:dataValidations count="2">
     <x:dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:C1000">
+      <x:formula1>"自媒体,官网留言,自主注册,渠道介绍,企查查,客源汇,公众号,地推,其他"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="D2:D1000">
       <x:formula1>"名单,线索,商机,成交,公海"</x:formula1>
-    </x:dataValidation>
-    <x:dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F2:F1000">
-      <x:formula1>"自媒体,官网留言,自主注册,渠道介绍,企查查,客源汇,公众号,地推,其他"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -17511,34 +17511,34 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="22" t="str">
+        <x:v>渠道来源</x:v>
+      </x:c>
+      <x:c r="B6" s="23" t="str">
+        <x:v>可选：自媒体、官网留言、自主注册、渠道介绍、企查查、客源汇、公众号、地推、其他。系统设置中新增的渠道也可以直接填写。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="22" t="str">
         <x:v>状态</x:v>
       </x:c>
-      <x:c r="B6" s="23" t="str">
+      <x:c r="B7" s="23" t="str">
         <x:v>可选：名单、线索、商机、成交、公海。为空时按当前导入入口处理；选择公海时不需要默认跟进人。</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="22" t="str">
+    <x:row r="8">
+      <x:c r="A8" s="22" t="str">
         <x:v>城市</x:v>
       </x:c>
-      <x:c r="B7" s="23" t="str">
+      <x:c r="B8" s="23" t="str">
         <x:v>建议填写；如留空系统会优先从客户地址中提取。</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="22" t="str">
+    <x:row r="9">
+      <x:c r="A9" s="22" t="str">
         <x:v>客户地址</x:v>
       </x:c>
-      <x:c r="B8" s="23" t="str">
+      <x:c r="B9" s="23" t="str">
         <x:v>建议填写完整省市区和街道；公海可先留空，系统会标记待补地址，暂不显示地图灰点。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="22" t="str">
-        <x:v>渠道来源</x:v>
-      </x:c>
-      <x:c r="B9" s="23" t="str">
-        <x:v>可选：自媒体、官网留言、自主注册、渠道介绍、企查查、客源汇、公众号、地推、其他。系统设置中新增的渠道也可以直接填写。</x:v>
       </x:c>
     </x:row>
     <x:row r="10">

</xml_diff>